<commit_message>
Minor changes to scripting
</commit_message>
<xml_diff>
--- a/data/processed/instances/graphs/voll_table.xlsx
+++ b/data/processed/instances/graphs/voll_table.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FarhadBillimoria\OneDrive - Aurora Energy Research\Documents\Personal\Endog_demand_AI\pyai\data\processed\instances\graphs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://auroraer-my.sharepoint.com/personal/farhad_billimoria_auroraer_com/Documents/Documents/Personal/Endog_demand_AI/pyai/data/processed/instances/graphs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{CAB09122-BA78-4B64-9D93-7876A1E75D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:9_{CAB09122-BA78-4B64-9D93-7876A1E75D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB1F3F9A-CEED-4547-A828-09E2260F19F4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EE0F3C9F-908A-40EA-9D05-B964B7DDA71B}"/>
   </bookViews>
@@ -18,12 +18,25 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">voll_box_panel_by_gpu_ondemand_!$A$1:$G$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="113">
   <si>
     <t>gpu_model_clean</t>
   </si>
@@ -851,10 +864,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1310,10 +1323,10 @@
       <c r="G3">
         <v>3502.7864855450998</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="L3" s="2"/>
+      <c r="L3" s="3"/>
       <c r="O3" t="s">
         <v>104</v>
       </c>
@@ -1401,6 +1414,9 @@
         <f>"$"&amp;S5&amp;" - "&amp;T5&amp;"/MWh"</f>
         <v>$500 - 1700/MWh</v>
       </c>
+      <c r="N5" t="s">
+        <v>11</v>
+      </c>
       <c r="O5">
         <f>ROUND(MEDIAN($D$5:$E$18),-2)</f>
         <v>2600</v>
@@ -1453,6 +1469,9 @@
         <f t="shared" ref="L6:L8" si="1">"$"&amp;S6&amp;" - "&amp;T6&amp;"/MWh"</f>
         <v>$1100 - 3100/MWh</v>
       </c>
+      <c r="N6" t="s">
+        <v>26</v>
+      </c>
       <c r="O6">
         <f>ROUND(MEDIAN($D$67:$E$77),-2)</f>
         <v>8100</v>
@@ -1505,6 +1524,9 @@
         <f t="shared" si="1"/>
         <v>$1800 - 5700/MWh</v>
       </c>
+      <c r="N7" t="s">
+        <v>8</v>
+      </c>
       <c r="O7">
         <f>ROUND(MEDIAN($D$19:$E$66),-2)</f>
         <v>8300</v>
@@ -1556,6 +1578,9 @@
       <c r="L8" s="1" t="str">
         <f t="shared" si="1"/>
         <v>$2400 - 3300/MWh</v>
+      </c>
+      <c r="N8" t="s">
+        <v>98</v>
       </c>
       <c r="O8">
         <f>ROUND(MEDIAN($D$2:$E$4),-2)</f>

</xml_diff>